<commit_message>
data: 更新配置表 — SummonChessTable / SummonChessSkillTable / ResourceConfigTable
- SummonChessSkillTable 新增/调整技能字段
- ResourceConfigTable 新增 InteractTip 等资源条目
</commit_message>
<xml_diff>
--- a/AAAGameData/DataTables/ResourceConfigTable.xlsx
+++ b/AAAGameData/DataTables/ResourceConfigTable.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29868" windowHeight="14855"/>
+    <workbookView windowWidth="28800" windowHeight="11925"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="268">
   <si>
     <t>#</t>
   </si>
@@ -56,7 +56,12 @@
     <t>资源ID</t>
   </si>
   <si>
-    <t>1：Assets/AAAGame/Sprites/2：Assets/AAAGame/Prefabs/3：Assets/AAAGame/Entities/4：Assets/AAAGame/Materials/5：Assets/AAAGame/Textures/6：Assets/AAAGame/Config/备注：大型资源和通用资源放这里</t>
+    <t>1：Assets/AAAGame/Sprites/
+2：Assets/AAAGame/Prefabs/
+3：Assets/AAAGame/Prefabs/Entity/
+4：Assets/AAAGame/Materials/
+5：Assets/AAAGame/Textures/
+6：Assets/AAAGame/Config/</t>
   </si>
   <si>
     <t>资源类型：1 = Sprite（图片）2 = Prefab（预制体）3 = Effect（特效）4 = Material（材质）5 = Texture（纹理）6 = ScriptableObject（配置文件）</t>
@@ -611,6 +616,12 @@
     <t>伤害飘字预制体</t>
   </si>
   <si>
+    <t>InteractTip</t>
+  </si>
+  <si>
+    <t>交互提示预制体</t>
+  </si>
+  <si>
     <t>Combat/BattleArena</t>
   </si>
   <si>
@@ -650,7 +661,13 @@
     <t>SummonChessEffect/Change_Skill2</t>
   </si>
   <si>
-    <t>嫦娥大招特效</t>
+    <t>嫦娥大招法阵预制体</t>
+  </si>
+  <si>
+    <t>SummonChessEffect/Change_Skill2_Projectile</t>
+  </si>
+  <si>
+    <t>嫦娥大招法阵生成的投射物</t>
   </si>
   <si>
     <t>Skills/SkillParamRegistry</t>
@@ -1783,8 +1800,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F132"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="5"/>
+  <dimension ref="A1:F134"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
@@ -1841,7 +1858,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" ht="86.4" spans="1:6">
+    <row r="4" ht="81" spans="1:6">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -3352,11 +3369,11 @@
     <row r="98" ht="15" customHeight="1" spans="1:6">
       <c r="A98" s="1"/>
       <c r="B98" s="1">
-        <v>2901</v>
+        <v>2402</v>
       </c>
       <c r="C98" s="1"/>
       <c r="D98" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E98" s="1" t="s">
         <v>194</v>
@@ -3368,11 +3385,11 @@
     <row r="99" ht="15" customHeight="1" spans="1:6">
       <c r="A99" s="1"/>
       <c r="B99" s="1">
-        <v>3001</v>
+        <v>2901</v>
       </c>
       <c r="C99" s="1"/>
       <c r="D99" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E99" s="1" t="s">
         <v>196</v>
@@ -3384,7 +3401,7 @@
     <row r="100" ht="15" customHeight="1" spans="1:6">
       <c r="A100" s="1"/>
       <c r="B100" s="1">
-        <v>3002</v>
+        <v>3001</v>
       </c>
       <c r="C100" s="1"/>
       <c r="D100" s="1">
@@ -3400,7 +3417,7 @@
     <row r="101" ht="15" customHeight="1" spans="1:6">
       <c r="A101" s="1"/>
       <c r="B101" s="1">
-        <v>3003</v>
+        <v>3002</v>
       </c>
       <c r="C101" s="1"/>
       <c r="D101" s="1">
@@ -3416,7 +3433,7 @@
     <row r="102" ht="15" customHeight="1" spans="1:6">
       <c r="A102" s="1"/>
       <c r="B102" s="1">
-        <v>3004</v>
+        <v>3003</v>
       </c>
       <c r="C102" s="1"/>
       <c r="D102" s="1">
@@ -3432,7 +3449,7 @@
     <row r="103" ht="15" customHeight="1" spans="1:6">
       <c r="A103" s="1"/>
       <c r="B103" s="1">
-        <v>3005</v>
+        <v>3004</v>
       </c>
       <c r="C103" s="1"/>
       <c r="D103" s="1">
@@ -3448,7 +3465,7 @@
     <row r="104" ht="15" customHeight="1" spans="1:6">
       <c r="A104" s="1"/>
       <c r="B104" s="1">
-        <v>3006</v>
+        <v>3005</v>
       </c>
       <c r="C104" s="1"/>
       <c r="D104" s="1">
@@ -3464,11 +3481,11 @@
     <row r="105" ht="15" customHeight="1" spans="1:6">
       <c r="A105" s="1"/>
       <c r="B105" s="1">
-        <v>6001</v>
+        <v>3006</v>
       </c>
       <c r="C105" s="1"/>
       <c r="D105" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E105" s="1" t="s">
         <v>208</v>
@@ -3480,11 +3497,11 @@
     <row r="106" ht="15" customHeight="1" spans="1:6">
       <c r="A106" s="1"/>
       <c r="B106" s="1">
-        <v>10001</v>
+        <v>3007</v>
       </c>
       <c r="C106" s="1"/>
       <c r="D106" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E106" s="1" t="s">
         <v>210</v>
@@ -3496,11 +3513,11 @@
     <row r="107" ht="15" customHeight="1" spans="1:6">
       <c r="A107" s="1"/>
       <c r="B107" s="1">
-        <v>10002</v>
+        <v>6001</v>
       </c>
       <c r="C107" s="1"/>
       <c r="D107" s="1">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E107" s="1" t="s">
         <v>212</v>
@@ -3512,7 +3529,7 @@
     <row r="108" ht="15" customHeight="1" spans="1:6">
       <c r="A108" s="1"/>
       <c r="B108" s="1">
-        <v>10003</v>
+        <v>10001</v>
       </c>
       <c r="C108" s="1"/>
       <c r="D108" s="1">
@@ -3528,7 +3545,7 @@
     <row r="109" ht="15" customHeight="1" spans="1:6">
       <c r="A109" s="1"/>
       <c r="B109" s="1">
-        <v>10004</v>
+        <v>10002</v>
       </c>
       <c r="C109" s="1"/>
       <c r="D109" s="1">
@@ -3544,7 +3561,7 @@
     <row r="110" ht="15" customHeight="1" spans="1:6">
       <c r="A110" s="1"/>
       <c r="B110" s="1">
-        <v>10101</v>
+        <v>10003</v>
       </c>
       <c r="C110" s="1"/>
       <c r="D110" s="1">
@@ -3560,7 +3577,7 @@
     <row r="111" ht="15" customHeight="1" spans="1:6">
       <c r="A111" s="1"/>
       <c r="B111" s="1">
-        <v>10102</v>
+        <v>10004</v>
       </c>
       <c r="C111" s="1"/>
       <c r="D111" s="1">
@@ -3576,7 +3593,7 @@
     <row r="112" ht="15" customHeight="1" spans="1:6">
       <c r="A112" s="1"/>
       <c r="B112" s="1">
-        <v>10103</v>
+        <v>10101</v>
       </c>
       <c r="C112" s="1"/>
       <c r="D112" s="1">
@@ -3592,7 +3609,7 @@
     <row r="113" ht="15" customHeight="1" spans="1:6">
       <c r="A113" s="1"/>
       <c r="B113" s="1">
-        <v>10201</v>
+        <v>10102</v>
       </c>
       <c r="C113" s="1"/>
       <c r="D113" s="1">
@@ -3608,7 +3625,7 @@
     <row r="114" ht="15" customHeight="1" spans="1:6">
       <c r="A114" s="1"/>
       <c r="B114" s="1">
-        <v>10202</v>
+        <v>10103</v>
       </c>
       <c r="C114" s="1"/>
       <c r="D114" s="1">
@@ -3624,7 +3641,7 @@
     <row r="115" ht="15" customHeight="1" spans="1:6">
       <c r="A115" s="1"/>
       <c r="B115" s="1">
-        <v>10203</v>
+        <v>10201</v>
       </c>
       <c r="C115" s="1"/>
       <c r="D115" s="1">
@@ -3640,7 +3657,7 @@
     <row r="116" ht="15" customHeight="1" spans="1:6">
       <c r="A116" s="1"/>
       <c r="B116" s="1">
-        <v>15001</v>
+        <v>10202</v>
       </c>
       <c r="C116" s="1"/>
       <c r="D116" s="1">
@@ -3656,7 +3673,7 @@
     <row r="117" ht="15" customHeight="1" spans="1:6">
       <c r="A117" s="1"/>
       <c r="B117" s="1">
-        <v>15002</v>
+        <v>10203</v>
       </c>
       <c r="C117" s="1"/>
       <c r="D117" s="1">
@@ -3672,7 +3689,7 @@
     <row r="118" ht="15" customHeight="1" spans="1:6">
       <c r="A118" s="1"/>
       <c r="B118" s="1">
-        <v>15003</v>
+        <v>15001</v>
       </c>
       <c r="C118" s="1"/>
       <c r="D118" s="1">
@@ -3688,7 +3705,7 @@
     <row r="119" ht="15" customHeight="1" spans="1:6">
       <c r="A119" s="1"/>
       <c r="B119" s="1">
-        <v>15005</v>
+        <v>15002</v>
       </c>
       <c r="C119" s="1"/>
       <c r="D119" s="1">
@@ -3704,7 +3721,7 @@
     <row r="120" ht="15" customHeight="1" spans="1:6">
       <c r="A120" s="1"/>
       <c r="B120" s="1">
-        <v>15007</v>
+        <v>15003</v>
       </c>
       <c r="C120" s="1"/>
       <c r="D120" s="1">
@@ -3720,7 +3737,7 @@
     <row r="121" ht="15" customHeight="1" spans="1:6">
       <c r="A121" s="1"/>
       <c r="B121" s="1">
-        <v>15008</v>
+        <v>15005</v>
       </c>
       <c r="C121" s="1"/>
       <c r="D121" s="1">
@@ -3736,7 +3753,7 @@
     <row r="122" ht="15" customHeight="1" spans="1:6">
       <c r="A122" s="1"/>
       <c r="B122" s="1">
-        <v>15009</v>
+        <v>15007</v>
       </c>
       <c r="C122" s="1"/>
       <c r="D122" s="1">
@@ -3752,7 +3769,7 @@
     <row r="123" ht="15" customHeight="1" spans="1:6">
       <c r="A123" s="1"/>
       <c r="B123" s="1">
-        <v>19002</v>
+        <v>15008</v>
       </c>
       <c r="C123" s="1"/>
       <c r="D123" s="1">
@@ -3768,7 +3785,7 @@
     <row r="124" ht="15" customHeight="1" spans="1:6">
       <c r="A124" s="1"/>
       <c r="B124" s="1">
-        <v>19003</v>
+        <v>15009</v>
       </c>
       <c r="C124" s="1"/>
       <c r="D124" s="1">
@@ -3784,7 +3801,7 @@
     <row r="125" ht="15" customHeight="1" spans="1:6">
       <c r="A125" s="1"/>
       <c r="B125" s="1">
-        <v>19004</v>
+        <v>19002</v>
       </c>
       <c r="C125" s="1"/>
       <c r="D125" s="1">
@@ -3800,7 +3817,7 @@
     <row r="126" ht="15" customHeight="1" spans="1:6">
       <c r="A126" s="1"/>
       <c r="B126" s="1">
-        <v>19012</v>
+        <v>19003</v>
       </c>
       <c r="C126" s="1"/>
       <c r="D126" s="1">
@@ -3816,7 +3833,7 @@
     <row r="127" ht="15" customHeight="1" spans="1:6">
       <c r="A127" s="1"/>
       <c r="B127" s="1">
-        <v>19013</v>
+        <v>19004</v>
       </c>
       <c r="C127" s="1"/>
       <c r="D127" s="1">
@@ -3832,7 +3849,7 @@
     <row r="128" ht="15" customHeight="1" spans="1:6">
       <c r="A128" s="1"/>
       <c r="B128" s="1">
-        <v>19014</v>
+        <v>19012</v>
       </c>
       <c r="C128" s="1"/>
       <c r="D128" s="1">
@@ -3848,7 +3865,7 @@
     <row r="129" ht="15" customHeight="1" spans="1:6">
       <c r="A129" s="1"/>
       <c r="B129" s="1">
-        <v>19022</v>
+        <v>19013</v>
       </c>
       <c r="C129" s="1"/>
       <c r="D129" s="1">
@@ -3864,7 +3881,7 @@
     <row r="130" ht="15" customHeight="1" spans="1:6">
       <c r="A130" s="1"/>
       <c r="B130" s="1">
-        <v>19023</v>
+        <v>19014</v>
       </c>
       <c r="C130" s="1"/>
       <c r="D130" s="1">
@@ -3880,7 +3897,7 @@
     <row r="131" ht="15" customHeight="1" spans="1:6">
       <c r="A131" s="1"/>
       <c r="B131" s="1">
-        <v>19024</v>
+        <v>19022</v>
       </c>
       <c r="C131" s="1"/>
       <c r="D131" s="1">
@@ -3893,18 +3910,50 @@
         <v>261</v>
       </c>
     </row>
-    <row r="132" spans="1:6">
-      <c r="B132">
+    <row r="132" ht="15" customHeight="1" spans="1:6">
+      <c r="A132" s="1"/>
+      <c r="B132" s="1">
+        <v>19023</v>
+      </c>
+      <c r="C132" s="1"/>
+      <c r="D132" s="1">
+        <v>1</v>
+      </c>
+      <c r="E132" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="F132" s="1" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="133" ht="15" customHeight="1" spans="1:6">
+      <c r="A133" s="1"/>
+      <c r="B133" s="1">
+        <v>19024</v>
+      </c>
+      <c r="C133" s="1"/>
+      <c r="D133" s="1">
+        <v>1</v>
+      </c>
+      <c r="E133" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="F133" s="1" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6">
+      <c r="B134">
         <v>11001</v>
       </c>
-      <c r="D132">
-        <v>1</v>
-      </c>
-      <c r="E132" t="s">
-        <v>262</v>
-      </c>
-      <c r="F132" t="s">
-        <v>263</v>
+      <c r="D134">
+        <v>1</v>
+      </c>
+      <c r="E134" t="s">
+        <v>266</v>
+      </c>
+      <c r="F134" t="s">
+        <v>267</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: DataTable 配置表更新 — SummonerTable 新增 HeadImgId，新增 ExpRuleTable
- SummonerTable 新增 HeadImgId 字段（召唤师头像资源 ID）
- 新增 ExpRuleTable（经验规则表，PlayerExpManager 使用）
- 同步更新 PlayerDataTable/ResourceConfigTable/SummonChessTable 配置数据
</commit_message>
<xml_diff>
--- a/AAAGameData/DataTables/ResourceConfigTable.xlsx
+++ b/AAAGameData/DataTables/ResourceConfigTable.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="388">
   <si>
     <t>#</t>
   </si>
@@ -1167,6 +1167,30 @@
   </si>
   <si>
     <t>敌人测试预制体</t>
+  </si>
+  <si>
+    <t>Summoner/召唤师头像/狂战士.png</t>
+  </si>
+  <si>
+    <t>狂战士头像</t>
+  </si>
+  <si>
+    <t>Summoner/召唤师头像/术士.png</t>
+  </si>
+  <si>
+    <t>术士头像</t>
+  </si>
+  <si>
+    <t>Summoner/召唤师头像/混沌.png</t>
+  </si>
+  <si>
+    <t>混沌头像</t>
+  </si>
+  <si>
+    <t>Summoner/召唤师头像/德鲁伊.png</t>
+  </si>
+  <si>
+    <t>德鲁伊头像</t>
   </si>
 </sst>
 </file>
@@ -2138,7 +2162,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F189"/>
+  <dimension ref="A1:F193"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -5182,6 +5206,62 @@
         <v>379</v>
       </c>
     </row>
+    <row r="190" spans="1:6">
+      <c r="B190">
+        <v>1155</v>
+      </c>
+      <c r="D190">
+        <v>1</v>
+      </c>
+      <c r="E190" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="F190" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6">
+      <c r="B191">
+        <v>1156</v>
+      </c>
+      <c r="D191">
+        <v>1</v>
+      </c>
+      <c r="E191" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="F191" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="192" spans="1:6">
+      <c r="B192">
+        <v>1157</v>
+      </c>
+      <c r="D192">
+        <v>1</v>
+      </c>
+      <c r="E192" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="F192" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="193" spans="2:6">
+      <c r="B193">
+        <v>1158</v>
+      </c>
+      <c r="D193">
+        <v>1</v>
+      </c>
+      <c r="E193" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="F193" t="s">
+        <v>387</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>